<commit_message>
Fill all PLO columns using only outcomes from the program specification
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DT1PLGbC6KyR6eFwVtGDq3
</commit_message>
<xml_diff>
--- a/PLOs_التصميم_الجرافيكي.xlsx
+++ b/PLOs_التصميم_الجرافيكي.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="67">
+  <fonts count="66">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -446,14 +446,8 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -506,11 +500,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFBE2D5"/>
         <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1041,7 +1030,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="254">
+  <cellXfs count="250">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1769,20 +1758,8 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1791,71 +1768,6 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors/>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Claude</author>
-  </authors>
-  <commentList>
-    <comment ref="H3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مقررات تاريخ التصميم الجرافيكي (206 جفك) وتاريخ الفنون القديمة (102 فنن) ونظريات التصميم (211 تيم).</t>
-      </text>
-    </comment>
-    <comment ref="J3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مقررات تصميم تجربة المستخدم (312 جفك) وواجهة المستخدم (336 جفك) والتصميم التفاعلي (414 جفك) وتصميم الحركة (332 جفك).</t>
-      </text>
-    </comment>
-    <comment ref="P3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مقرر مدخل إلى النقد والتذوق الفني (103 فنن) وهدف البرنامج الثالث (تطوير القدرات الإبداعية والاستقصاء).</t>
-      </text>
-    </comment>
-    <comment ref="T3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مقررات مهارات الاتصال في الفنون (241 تصل) ومهارات الكتابة (100 عرب) وأساسيات تصميم التواصل البصري (205 جفك).</t>
-      </text>
-    </comment>
-    <comment ref="X3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مخرج المعرفة (ع2) ومقررات مدخل إلى برامج وتطبيقات التصميم (207 تيم) وتصميم المواقع (318 جفك).</t>
-      </text>
-    </comment>
-    <comment ref="Z3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مقررات التصميم ثلاثي الأبعاد (320 جفك) وتصميم المغلفات (330 جفك) وتجهيزات البرنامج (معمل طباعة 3D، استديو تصوير).</t>
-      </text>
-    </comment>
-    <comment ref="AD3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مقررات البحث في التصميم الجرافيكي (310 جفك) ومشروع بحثي في التصميم (410 جفك) ومخرج المعرفة (ع3).</t>
-      </text>
-    </comment>
-    <comment ref="AF3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مخرج القيم (ق3) ومقررات مشروع التخرج (420 جفك) والتدريب التعاوني (450 جفك).</t>
-      </text>
-    </comment>
-    <comment ref="AH3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى رسالة البرنامج وهدفيه الرابع والسادس (مواكبة المستجدات والتعامل مع التطورات التقنية وفق احتياجات سوق العمل).</t>
-      </text>
-    </comment>
-    <comment ref="AN3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى رسالة البرنامج (كوادر قادرة على مواكبة التطور التقني التكنولوجي) والهدف الخامس.</t>
-      </text>
-    </comment>
-    <comment ref="AP3" authorId="0" shapeId="0">
-      <text>
-        <t>مخرج مقترح: لا يوجد في توصيف البرنامج مخرج مطابق مباشرة لهذا المعيار، وتمت صياغته استناداً إلى مخرج المهارات (م4) والهدف الخامس (تحسين جودة الحياة) ومقرر الفن والمجتمع (102 فاد).</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2552,7 +2464,7 @@
       <c r="AU2" s="43" t="n"/>
     </row>
     <row r="3" ht="140" customHeight="1">
-      <c r="A3" s="84" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>برنامج التصميم الجرافيكي (بكالوريوس) - كلية الفنون</t>
         </is>
@@ -2581,17 +2493,17 @@
       <c r="G3" s="248" t="n">
         <v>0.75</v>
       </c>
-      <c r="H3" s="249" t="inlineStr">
+      <c r="H3" s="39" t="inlineStr">
         <is>
-          <t>يصف مراحل تطور التصميم الجرافيكي والفنون وأبرز مدارسها وروادها.</t>
+          <t>(ع1) يتعرف على المفاهيم والنظريات والاتجاهات الفنية في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
       <c r="I3" s="248" t="n">
         <v>0.75</v>
       </c>
-      <c r="J3" s="250" t="inlineStr">
+      <c r="J3" s="84" t="inlineStr">
         <is>
-          <t>يشرح مبادئ تصميم تجربة المستخدم وواجهات الاستخدام والتصميم التفاعلي والحركي.</t>
+          <t>(ع2) يستعرض خصائص الخامات الرقمية والأدوات والتطبيقات التقنية وطرق استخدامها.</t>
         </is>
       </c>
       <c r="K3" s="248" t="n">
@@ -2610,15 +2522,15 @@
           <t>(م2) يطبق المفاهيم والمهارات والاستراتيجيات والنظريات في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
-      <c r="O3" s="251" t="n">
+      <c r="O3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="P3" s="250" t="inlineStr">
+      <c r="P3" s="84" t="inlineStr">
         <is>
-          <t>يحلل ويقيّم الأعمال التصميمية نقدياً وفق أسس التذوق الفني ومعايير التصميم.</t>
+          <t>(م4) ينتج أعمال وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
         </is>
       </c>
-      <c r="Q3" s="251" t="n">
+      <c r="Q3" s="249" t="n">
         <v>0.75</v>
       </c>
       <c r="R3" s="84" t="inlineStr">
@@ -2626,15 +2538,15 @@
           <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
         </is>
       </c>
-      <c r="S3" s="251" t="n">
+      <c r="S3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="T3" s="250" t="inlineStr">
+      <c r="T3" s="84" t="inlineStr">
         <is>
-          <t>يعرض أفكاره وحلوله التصميمية بصرياً وشفهياً وكتابياً بوضوح لمختلف الفئات المستهدفة.</t>
+          <t>(م4) ينتج أعمال وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
         </is>
       </c>
-      <c r="U3" s="251" t="n">
+      <c r="U3" s="249" t="n">
         <v>0.75</v>
       </c>
       <c r="V3" s="84" t="inlineStr">
@@ -2642,55 +2554,55 @@
           <t>(م3) يصمم باستخدام التقنيات والبرامج لإنتاج أعمال تساهم في تعزيز الهوية الوطنية والثقافية.</t>
         </is>
       </c>
-      <c r="W3" s="251" t="n">
+      <c r="W3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="X3" s="250" t="inlineStr">
+      <c r="X3" s="84" t="inlineStr">
         <is>
-          <t>يوظف برامج وتطبيقات التصميم الرقمي في إنتاج تصاميم مطبوعة ورقمية وتفاعلية.</t>
+          <t>(م2) يطبق المفاهيم والمهارات والاستراتيجيات والنظريات في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
-      <c r="Y3" s="251" t="n">
+      <c r="Y3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="Z3" s="252" t="inlineStr">
+      <c r="Z3" s="46" t="inlineStr">
         <is>
-          <t>يستخدم تقنيات النمذجة ثلاثية الأبعاد والطباعة والتصوير في تنفيذ المنتجات التصميمية.</t>
+          <t>(م1) يقارن بين الأدوات والأساليب التقنية والمعرفية في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
-      <c r="AA3" s="251" t="n">
+      <c r="AA3" s="249" t="n">
         <v>0.75</v>
       </c>
       <c r="AB3" s="84" t="inlineStr">
         <is>
-          <t>(م4) ينتج أعمالاً وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
+          <t>(م4) ينتج أعمال وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
         </is>
       </c>
       <c r="AC3" s="248" t="n">
         <v>0.75</v>
       </c>
-      <c r="AD3" s="250" t="inlineStr">
+      <c r="AD3" s="84" t="inlineStr">
         <is>
-          <t>يوظف مناهج البحث العلمي في إعداد بحث أو مشروع بحثي في مجال التصميم الجرافيكي.</t>
+          <t>(م4) ينتج أعمال وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
         </is>
       </c>
       <c r="AE3" s="248" t="n">
         <v>0.75</v>
       </c>
-      <c r="AF3" s="250" t="inlineStr">
+      <c r="AF3" s="84" t="inlineStr">
         <is>
-          <t>يتحمل مسؤولية أداء المهام والأدوار القيادية ضمن فرق العمل في المشاريع التصميمية.</t>
+          <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
         </is>
       </c>
-      <c r="AG3" s="251" t="n">
+      <c r="AG3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="AH3" s="250" t="inlineStr">
+      <c r="AH3" s="84" t="inlineStr">
         <is>
-          <t>يبادر ويتكيف مع المستجدات والتطورات التقنية المتسارعة في مجال التصميم وسوق العمل.</t>
+          <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
         </is>
       </c>
-      <c r="AI3" s="251" t="n">
+      <c r="AI3" s="249" t="n">
         <v>0.75</v>
       </c>
       <c r="AJ3" s="84" t="inlineStr">
@@ -2698,7 +2610,7 @@
           <t>(ق1) يلتزم بالأخلاقيات المهنية والحقوق الفكرية في التصميم.</t>
         </is>
       </c>
-      <c r="AK3" s="251" t="n">
+      <c r="AK3" s="249" t="n">
         <v>0.75</v>
       </c>
       <c r="AL3" s="84" t="inlineStr">
@@ -2706,23 +2618,23 @@
           <t>(ق2) يقدر أهمية العمل اليدوي والتقني وارتباطه بالهوية الثقافية.</t>
         </is>
       </c>
-      <c r="AM3" s="251" t="n">
+      <c r="AM3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="AN3" s="250" t="inlineStr">
+      <c r="AN3" s="84" t="inlineStr">
         <is>
-          <t>يطور معارفه ومهاراته التصميمية ذاتياً وباستمرار لمواكبة التطور التقني.</t>
+          <t>(ق2) يقدر أهمية العمل اليدوي والتقني وارتباطه بالهوية الثقافية.</t>
         </is>
       </c>
-      <c r="AO3" s="251" t="n">
+      <c r="AO3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="AP3" s="250" t="inlineStr">
+      <c r="AP3" s="84" t="inlineStr">
         <is>
-          <t>يوظف مهاراته التصميمية في خدمة المجتمع والمبادرات التطوعية بما يسهم في تحسين جودة الحياة.</t>
+          <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
         </is>
       </c>
-      <c r="AQ3" s="251" t="n">
+      <c r="AQ3" s="249" t="n">
         <v>0.75</v>
       </c>
       <c r="AR3" s="43" t="n"/>
@@ -2753,11 +2665,6 @@
       <c r="AU4" s="43" t="n"/>
     </row>
     <row r="5" ht="69" customHeight="1">
-      <c r="A5" s="253" t="inlineStr">
-        <is>
-          <t>ملاحظة: الخلايا المظللة بالأصفر مخرجات مقترحة لعدم وجود مخرج مطابق في توصيف البرنامج (انظر التعليق على كل خلية). القيمة المستهدفة لجميع المخرجات 75% (حسب طلب المستخدم).</t>
-        </is>
-      </c>
       <c r="B5" s="39" t="n"/>
       <c r="C5" s="46" t="n"/>
       <c r="D5" s="39" t="n"/>
@@ -7294,7 +7201,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">

</xml_diff>

<commit_message>
Keep only strong or close PLO mappings; leave unmatched criteria blank
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DT1PLGbC6KyR6eFwVtGDq3
</commit_message>
<xml_diff>
--- a/PLOs_التصميم_الجرافيكي.xlsx
+++ b/PLOs_التصميم_الجرافيكي.xlsx
@@ -2493,22 +2493,9 @@
       <c r="G3" s="248" t="n">
         <v>0.75</v>
       </c>
-      <c r="H3" s="39" t="inlineStr">
-        <is>
-          <t>(ع1) يتعرف على المفاهيم والنظريات والاتجاهات الفنية في مجال التصميم الجرافيكي.</t>
-        </is>
-      </c>
-      <c r="I3" s="248" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J3" s="84" t="inlineStr">
-        <is>
-          <t>(ع2) يستعرض خصائص الخامات الرقمية والأدوات والتطبيقات التقنية وطرق استخدامها.</t>
-        </is>
-      </c>
-      <c r="K3" s="248" t="n">
-        <v>0.75</v>
-      </c>
+      <c r="H3" s="39" t="n"/>
+      <c r="I3" s="46" t="n"/>
+      <c r="K3" s="46" t="n"/>
       <c r="L3" s="39" t="inlineStr">
         <is>
           <t>(م1) يقارن بين الأدوات والأساليب التقنية والمعرفية في مجال التصميم الجرافيكي.</t>
@@ -2525,14 +2512,6 @@
       <c r="O3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="P3" s="84" t="inlineStr">
-        <is>
-          <t>(م4) ينتج أعمال وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
-        </is>
-      </c>
-      <c r="Q3" s="249" t="n">
-        <v>0.75</v>
-      </c>
       <c r="R3" s="84" t="inlineStr">
         <is>
           <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
@@ -2597,14 +2576,6 @@
       <c r="AG3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="AH3" s="84" t="inlineStr">
-        <is>
-          <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
-        </is>
-      </c>
-      <c r="AI3" s="249" t="n">
-        <v>0.75</v>
-      </c>
       <c r="AJ3" s="84" t="inlineStr">
         <is>
           <t>(ق1) يلتزم بالأخلاقيات المهنية والحقوق الفكرية في التصميم.</t>
@@ -2621,17 +2592,9 @@
       <c r="AM3" s="249" t="n">
         <v>0.75</v>
       </c>
-      <c r="AN3" s="84" t="inlineStr">
-        <is>
-          <t>(ق2) يقدر أهمية العمل اليدوي والتقني وارتباطه بالهوية الثقافية.</t>
-        </is>
-      </c>
-      <c r="AO3" s="249" t="n">
-        <v>0.75</v>
-      </c>
       <c r="AP3" s="84" t="inlineStr">
         <is>
-          <t>(ق3) يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
+          <t>(م4) ينتج أعمال وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
         </is>
       </c>
       <c r="AQ3" s="249" t="n">

</xml_diff>